<commit_message>
Finalize main set (229 items): wording and meaning duplicate checks, rebuilt sheets and Gemini inputs
</commit_message>
<xml_diff>
--- a/data/main/sheets/batch_01.xlsx
+++ b/data/main/sheets/batch_01.xlsx
@@ -467,19 +467,18 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_343</t>
+          <t xml:space="preserve">simple_python_289</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fetch player statistics of 'Zelda' on Switch for user 'Sam'.</t>
+          <t xml:space="preserve">Find concerts near me in Seattle that plays jazz music.</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">game = Zelda
-username = Sam
-platform = Switch</t>
+          <t xml:space="preserve">location = Seattle
+genre = jazz</t>
         </is>
       </c>
       <c r="D3" s="6"/>
@@ -491,18 +490,19 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_142</t>
+          <t xml:space="preserve">simple_python_163</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the humidity level in Miami, Florida in the upcoming 7 days?</t>
+          <t xml:space="preserve">Provide me with the property records of my house located at 123 main street, with parcel number 1234567890 in Santa Clara county. Include owners information in the response.</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">location = Miami, Florida
-days = 7</t>
+          <t xml:space="preserve">address = 123 main street
+parcel_number = 1234567890
+county = Santa Clara</t>
         </is>
       </c>
       <c r="D4" s="6"/>
@@ -514,19 +514,19 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_163</t>
+          <t xml:space="preserve">multiple_185</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provide me with the property records of my house located at 123 main street, with parcel number 1234567890 in Santa Clara county. Include owners information in the response.</t>
+          <t xml:space="preserve">Find the closest sushi restaurant with a patio in Boston.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">address = 123 main street
-parcel_number = 1234567890
-county = Santa Clara</t>
+          <t xml:space="preserve">location = Boston
+cuisine = sushi
+amenities = patio</t>
         </is>
       </c>
       <c r="D5" s="6"/>
@@ -538,19 +538,18 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_185</t>
+          <t xml:space="preserve">simple_python_228</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find the closest sushi restaurant with a patio in Boston.</t>
+          <t xml:space="preserve">Find three personality traits of people who like jogging.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">location = Boston
-cuisine = sushi
-amenities = patio</t>
+          <t xml:space="preserve">hobby = jogging
+trait_count = three</t>
         </is>
       </c>
       <c r="D6" s="6"/>
@@ -562,18 +561,18 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_228</t>
+          <t xml:space="preserve">multiple_54</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find three personality traits of people who like jogging.</t>
+          <t xml:space="preserve">Find out the historical dividend payments of Apple Inc for last five years.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">hobby = jogging
-trait_count = three</t>
+          <t xml:space="preserve">company = Apple Inc
+years = five</t>
         </is>
       </c>
       <c r="D7" s="6"/>
@@ -585,18 +584,19 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_54</t>
+          <t xml:space="preserve">simple_python_165</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find out the historical dividend payments of Apple Inc for last five years.</t>
+          <t xml:space="preserve">Retrieve cases from 2020 about theft crimes in Los Angeles, California</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">company = Apple Inc
-years = five</t>
+          <t xml:space="preserve">year = 2020
+crime_type = theft
+location = Los Angeles, California</t>
         </is>
       </c>
       <c r="D8" s="6"/>
@@ -608,19 +608,18 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_165</t>
+          <t xml:space="preserve">simple_python_66</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retrieve cases from 2020 about theft crimes in Los Angeles, California</t>
+          <t xml:space="preserve">Get me data on average precipitation in the Amazon rainforest for the last six months.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">year = 2020
-crime_type = theft
-location = Los Angeles, California</t>
+          <t xml:space="preserve">location = Amazon rainforest
+time_frame = six months</t>
         </is>
       </c>
       <c r="D9" s="6"/>
@@ -632,18 +631,18 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_66</t>
+          <t xml:space="preserve">multiple_56</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Get me data on average precipitation in the Amazon rainforest for the last six months.</t>
+          <t xml:space="preserve">Find the average closing price of Apple stock in the past 60 days</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">location = Amazon rainforest
-time_frame = six months</t>
+          <t xml:space="preserve">company = Apple
+days = 60</t>
         </is>
       </c>
       <c r="D10" s="6"/>
@@ -655,18 +654,18 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_56</t>
+          <t xml:space="preserve">simple_python_280</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find the average closing price of Apple stock in the past 60 days</t>
+          <t xml:space="preserve">Find an acoustic instrument within my budget of $1000.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">company = Apple
-days = 60</t>
+          <t xml:space="preserve">budget = 1000
+type = acoustic</t>
         </is>
       </c>
       <c r="D11" s="6"/>
@@ -678,18 +677,18 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_280</t>
+          <t xml:space="preserve">multiple_60</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find an acoustic instrument within my budget of $1000.</t>
+          <t xml:space="preserve">What will be the humidity and temperature for New York City after 7 days?</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">budget = 1000
-type = acoustic</t>
+          <t xml:space="preserve">location = New York City
+days = 7</t>
         </is>
       </c>
       <c r="D12" s="6"/>
@@ -701,18 +700,17 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_60</t>
+          <t xml:space="preserve">simple_python_310</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What will be the humidity and temperature for New York City after 7 days?</t>
+          <t xml:space="preserve">What are the career stats of basketball player LeBron James?</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">location = New York City
-days = 7</t>
+          <t xml:space="preserve">player_name = LeBron James</t>
         </is>
       </c>
       <c r="D13" s="6"/>
@@ -724,17 +722,18 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_310</t>
+          <t xml:space="preserve">multiple_178</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What are the career stats of basketball player LeBron James?</t>
+          <t xml:space="preserve">Find a Card of rank 'Queen' and suit 'Hearts' in the deck.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">player_name = LeBron James</t>
+          <t xml:space="preserve">rank = Queen
+suit = Hearts</t>
         </is>
       </c>
       <c r="D14" s="6"/>
@@ -746,18 +745,19 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_178</t>
+          <t xml:space="preserve">simple_python_237</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find a Card of rank 'Queen' and suit 'Hearts' in the deck.</t>
+          <t xml:space="preserve">Get historical GDP data for United States from 1960 to 2000.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">rank = Queen
-suit = Hearts</t>
+          <t xml:space="preserve">country = United States
+start_year = 1960
+end_year = 2000</t>
         </is>
       </c>
       <c r="D15" s="6"/>
@@ -769,18 +769,17 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_200</t>
+          <t xml:space="preserve">simple_python_245</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">How much CO2 is produced annually by a gas-fueled car that travels 12,000 miles per year, with fuel efficiency of 25 MPG ?</t>
+          <t xml:space="preserve">Who discovered radium?</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">distance = 12,000
-fuel_type = gas</t>
+          <t xml:space="preserve">element_name = radium</t>
         </is>
       </c>
       <c r="D16" s="6"/>
@@ -792,17 +791,20 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_172</t>
+          <t xml:space="preserve">multiple_166</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">How to obtain the detailed case information of the 'R vs Adams' legal case?</t>
+          <t xml:space="preserve">Find me a classical concert this weekend in Los Angeles with cheap tickets.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">case_id = R vs Adams</t>
+          <t xml:space="preserve">genre = classical
+location = Los Angeles
+date = this weekend
+price_range = cheap</t>
         </is>
       </c>
       <c r="D17" s="6"/>
@@ -814,20 +816,18 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_166</t>
+          <t xml:space="preserve">simple_python_175</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find me a classical concert this weekend in Los Angeles with cheap tickets.</t>
+          <t xml:space="preserve">How many months of experience a Lawyer John Doe has on handling Bankruptcy cases.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">genre = classical
-location = Los Angeles
-date = this weekend
-price_range = cheap</t>
+          <t xml:space="preserve">name = John Doe
+law_type = Bankruptcy</t>
         </is>
       </c>
       <c r="D18" s="6"/>
@@ -839,18 +839,19 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_175</t>
+          <t xml:space="preserve">multiple_165</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many months of experience a Lawyer John Doe has on handling Bankruptcy cases.</t>
+          <t xml:space="preserve">Find the price of a used Gibson Les Paul guitar in excellent condition in the Chicago area.</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">name = John Doe
-law_type = Bankruptcy</t>
+          <t xml:space="preserve">model = Gibson Les Paul
+condition = excellent
+location = Chicago area</t>
         </is>
       </c>
       <c r="D19" s="6"/>
@@ -862,19 +863,18 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_165</t>
+          <t xml:space="preserve">simple_python_233</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find the price of a used Gibson Les Paul guitar in excellent condition in the Chicago area.</t>
+          <t xml:space="preserve">When did the Treaty of Tordesillas take place? Put it in the format of YYYY.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">model = Gibson Les Paul
-condition = excellent
-location = Chicago area</t>
+          <t xml:space="preserve">event_name = Treaty of Tordesillas
+format = YYYY</t>
         </is>
       </c>
       <c r="D20" s="6"/>
@@ -886,18 +886,18 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_233</t>
+          <t xml:space="preserve">simple_python_290</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">When did the Treaty of Tordesillas take place? Put it in the format of YYYY.</t>
+          <t xml:space="preserve">What's the timing and location for The Weeknd's concert happening in December?</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">event_name = Treaty of Tordesillas
-format = YYYY</t>
+          <t xml:space="preserve">artist = The Weeknd
+month = December</t>
         </is>
       </c>
       <c r="D21" s="6"/>
@@ -909,18 +909,17 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_290</t>
+          <t xml:space="preserve">multiple_22</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the timing and location for The Weeknd's concert happening in December?</t>
+          <t xml:space="preserve">What is the record for the most points scored by a single player in an NBA game?</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">artist = The Weeknd
-month = December</t>
+          <t xml:space="preserve">league = NBA</t>
         </is>
       </c>
       <c r="D22" s="6"/>
@@ -932,17 +931,17 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_22</t>
+          <t xml:space="preserve">simple_python_324</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the record for the most points scored by a single player in an NBA game?</t>
+          <t xml:space="preserve">Find the score of last game for Los Angeles Lakers including its opponent name.</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">league = NBA</t>
+          <t xml:space="preserve">team = Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D23" s="6"/>
@@ -954,7 +953,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_355</t>
+          <t xml:space="preserve">multiple_183</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -965,7 +964,7 @@
       <c r="C24" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">website = Foodnetwork.com
-recipe = Beef Lasagna</t>
+recipe = Beef Lasagna Recipe</t>
         </is>
       </c>
       <c r="D24" s="6"/>
@@ -977,18 +976,19 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_183</t>
+          <t xml:space="preserve">simple_python_157</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many calories in the Beef Lasagna Recipe from Foodnetwork.com?</t>
+          <t xml:space="preserve">Find out if an individual John Doe with a birthday 01-01-1980 has any prior felony convictions in California.</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">website = Foodnetwork.com
-recipe = Beef Lasagna Recipe</t>
+          <t xml:space="preserve">full_name = John Doe
+birth_date = 01-01-1980
+state = California</t>
         </is>
       </c>
       <c r="D25" s="6"/>
@@ -1000,19 +1000,17 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_157</t>
+          <t xml:space="preserve">multiple_2</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find out if an individual John Doe with a birthday 01-01-1980 has any prior felony convictions in California.</t>
+          <t xml:space="preserve">What is the capital of Brazil?</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">full_name = John Doe
-birth_date = 01-01-1980
-state = California</t>
+          <t xml:space="preserve">country = Brazil</t>
         </is>
       </c>
       <c r="D26" s="6"/>
@@ -1024,17 +1022,18 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_2</t>
+          <t xml:space="preserve">simple_python_322</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the capital of Brazil?</t>
+          <t xml:space="preserve">Get the current ranking for Liverpool Football Club in the Premier League.</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">country = Brazil</t>
+          <t xml:space="preserve">team = Liverpool Football Club
+league = Premier League</t>
         </is>
       </c>
       <c r="D27" s="6"/>
@@ -1046,18 +1045,19 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_322</t>
+          <t xml:space="preserve">simple_python_170</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Get the current ranking for Liverpool Football Club in the Premier League.</t>
+          <t xml:space="preserve">Find a historical law case about fraud from 2010 to 2015.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">team = Liverpool Football Club
-league = Premier League</t>
+          <t xml:space="preserve">subject = fraud
+from_year = 2010
+to_year = 2015</t>
         </is>
       </c>
       <c r="D28" s="6"/>
@@ -1069,19 +1069,20 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_170</t>
+          <t xml:space="preserve">multiple_115</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find a historical law case about fraud from 2010 to 2015.</t>
+          <t xml:space="preserve">I want to find 5 restaurants nearby my location, Manhattan, offering Thai food and a vegan menu.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">subject = fraud
-from_year = 2010
-to_year = 2015</t>
+          <t xml:space="preserve">location = Manhattan
+food_type = Thai
+number = 5
+dietary_requirements = vegan</t>
         </is>
       </c>
       <c r="D29" s="6"/>
@@ -1093,20 +1094,18 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_115</t>
+          <t xml:space="preserve">simple_python_342</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">I want to find 5 restaurants nearby my location, Manhattan, offering Thai food and a vegan menu.</t>
+          <t xml:space="preserve">Find all multi-player games released in 2019 with an ESRB rating of 'Everyone</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">location = Manhattan
-food_type = Thai
-number = 5
-dietary_requirements = vegan</t>
+          <t xml:space="preserve">release_year = 2019
+ESRB_rating = Everyone</t>
         </is>
       </c>
       <c r="D30" s="6"/>
@@ -1118,18 +1117,17 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_342</t>
+          <t xml:space="preserve">multiple_73</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find all multi-player games released in 2019 with an ESRB rating of 'Everyone</t>
+          <t xml:space="preserve">Who was the founder of Buddhism and where was it originated?</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">release_year = 2019
-ESRB_rating = Everyone</t>
+          <t xml:space="preserve">religion = Buddhism</t>
         </is>
       </c>
       <c r="D31" s="6"/>
@@ -1141,17 +1139,20 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_73</t>
+          <t xml:space="preserve">simple_python_252</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who was the founder of Buddhism and where was it originated?</t>
+          <t xml:space="preserve">Find ten major historical events related to Christianity in the 16th century sort by importance.</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">religion = Buddhism</t>
+          <t xml:space="preserve">religion = Christianity
+century = 16
+sort_by = importance
+count = ten</t>
         </is>
       </c>
       <c r="D32" s="6"/>
@@ -1163,20 +1164,20 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_252</t>
+          <t xml:space="preserve">multiple_129</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find ten major historical events related to Christianity in the 16th century sort by importance.</t>
+          <t xml:space="preserve">Find the compound interest for an investment of $10000 with an annual interest rate of 5% compounded monthly for 5 years.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">religion = Christianity
-century = 16
-sort_by = importance
-count = ten</t>
+          <t xml:space="preserve">principal = 10000
+annual_rate = 5
+compounding_freq = monthly
+time_in_years = 5</t>
         </is>
       </c>
       <c r="D33" s="6"/>
@@ -1188,20 +1189,18 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_129</t>
+          <t xml:space="preserve">simple_python_58</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find the compound interest for an investment of $10000 with an annual interest rate of 5% compounded monthly for 5 years.</t>
+          <t xml:space="preserve">What is the function of ATP synthase in mitochondria?</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">principal = 10000
-annual_rate = 5
-compounding_freq = monthly
-time_in_years = 5</t>
+          <t xml:space="preserve">molecule = ATP synthase
+organelle = mitochondria</t>
         </is>
       </c>
       <c r="D34" s="6"/>
@@ -1213,18 +1212,19 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_58</t>
+          <t xml:space="preserve">simple_python_258</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the function of ATP synthase in mitochondria?</t>
+          <t xml:space="preserve">Mix yellow and blue colors and adjust the lightness level to 60 percent.</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">molecule = ATP synthase
-organelle = mitochondria</t>
+          <t xml:space="preserve">color1 = yellow
+color2 = blue
+lightness = 60</t>
         </is>
       </c>
       <c r="D35" s="6"/>
@@ -1236,19 +1236,19 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_258</t>
+          <t xml:space="preserve">multiple_145</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mix yellow and blue colors and adjust the lightness level to 60 percent.</t>
+          <t xml:space="preserve">How much CO2 is produced annually by a gas-fueled car that travels 12,000 miles per year with fuel efficiency 20 mpg?</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">color1 = yellow
-color2 = blue
-lightness = 60</t>
+          <t xml:space="preserve">distance = 12,000
+fuel_type = gas
+fuel_efficiency = 20</t>
         </is>
       </c>
       <c r="D36" s="6"/>
@@ -1260,19 +1260,19 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_145</t>
+          <t xml:space="preserve">simple_python_171</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">How much CO2 is produced annually by a gas-fueled car that travels 12,000 miles per year with fuel efficiency 20 mpg?</t>
+          <t xml:space="preserve">Fetch details of a law case with number 43403 in New York court for year 2018.</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">distance = 12,000
-fuel_type = gas
-fuel_efficiency = 20</t>
+          <t xml:space="preserve">case_number = 43403
+court = New York
+year = 2018</t>
         </is>
       </c>
       <c r="D37" s="6"/>
@@ -1284,19 +1284,18 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_171</t>
+          <t xml:space="preserve">multiple_134</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fetch details of a law case with number 43403 in New York court for year 2018.</t>
+          <t xml:space="preserve">Look up details of a felony crime record for case number CA123456 in San Diego County</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">case_number = 43403
-court = New York
-year = 2018</t>
+          <t xml:space="preserve">case_number = CA123456
+county = San Diego County</t>
         </is>
       </c>
       <c r="D38" s="6"/>
@@ -1308,18 +1307,17 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_134</t>
+          <t xml:space="preserve">simple_python_257</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Look up details of a felony crime record for case number CA123456 in San Diego County</t>
+          <t xml:space="preserve">Can you help me identify the basic RGB value of Sea Green color?</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">case_number = CA123456
-county = San Diego County</t>
+          <t xml:space="preserve">color_name = Sea Green</t>
         </is>
       </c>
       <c r="D39" s="6"/>
@@ -1331,17 +1329,18 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_257</t>
+          <t xml:space="preserve">multiple_172</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can you help me identify the basic RGB value of Sea Green color?</t>
+          <t xml:space="preserve">Find me the detailed profile of basketball player Lebron James</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">color_name = Sea Green</t>
+          <t xml:space="preserve">name = Lebron James
+sport = basketball</t>
         </is>
       </c>
       <c r="D40" s="6"/>
@@ -1353,18 +1352,19 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">multiple_172</t>
+          <t xml:space="preserve">simple_python_321</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Find me the detailed profile of basketball player Lebron James</t>
+          <t xml:space="preserve">What's the ranking of Barcelona in the 2021 La Liga season?</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">name = Lebron James
-sport = basketball</t>
+          <t xml:space="preserve">team = Barcelona
+league = La Liga
+season = 2021</t>
         </is>
       </c>
       <c r="D41" s="6"/>
@@ -1376,19 +1376,19 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">simple_python_321</t>
+          <t xml:space="preserve">simple_python_78</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the ranking of Barcelona in the 2021 La Liga season?</t>
+          <t xml:space="preserve">Get the average temperature in Austin for the next 3 days in Celsius.</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">team = Barcelona
-league = La Liga
-season = 2021</t>
+          <t xml:space="preserve">location = Austin
+days = 3
+temp_unit = Celsius</t>
         </is>
       </c>
       <c r="D42" s="6"/>

</xml_diff>